<commit_message>
Pick up current xlsx files
These were not update (I think since the introduction of the function
'compare_with_git()', because 'file.copy()' was missing the argument
'overwrite = TRUE'.

The JSON files are unchanged, showing that the relevant contents
of the xlsx files did not change.

Fixes #1
</commit_message>
<xml_diff>
--- a/data_generation/06_soil_sorption/acetamiprid_soil_sorption.xlsx
+++ b/data_generation/06_soil_sorption/acetamiprid_soil_sorption.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\soil_sorption\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\06_soil_sorption\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15683D10-B6D0-4632-A58D-18948BEB107F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9DF5A32-7623-48E5-AF73-E7F8AA07D377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="410" yWindow="520" windowWidth="28800" windowHeight="15410" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,36 +33,6 @@
     <t>soil_name</t>
   </si>
   <si>
-    <t>soil_ph</t>
-  </si>
-  <si>
-    <t>p_clay</t>
-  </si>
-  <si>
-    <t>p_sand</t>
-  </si>
-  <si>
-    <t>p_silt</t>
-  </si>
-  <si>
-    <t>p_om</t>
-  </si>
-  <si>
-    <t>p_oc</t>
-  </si>
-  <si>
-    <t>kd</t>
-  </si>
-  <si>
-    <t>koc</t>
-  </si>
-  <si>
-    <t>kf</t>
-  </si>
-  <si>
-    <t>kfoc</t>
-  </si>
-  <si>
     <t>n</t>
   </si>
   <si>
@@ -132,7 +102,37 @@
     <t>III</t>
   </si>
   <si>
-    <t>ph_medium</t>
+    <t>soil_pH</t>
+  </si>
+  <si>
+    <t>pH_medium</t>
+  </si>
+  <si>
+    <t>f_clay</t>
+  </si>
+  <si>
+    <t>f_sand</t>
+  </si>
+  <si>
+    <t>f_silt</t>
+  </si>
+  <si>
+    <t>f_om</t>
+  </si>
+  <si>
+    <t>f_oc</t>
+  </si>
+  <si>
+    <t>Kd</t>
+  </si>
+  <si>
+    <t>Koc</t>
+  </si>
+  <si>
+    <t>Kf</t>
+  </si>
+  <si>
+    <t>Kfoc</t>
   </si>
 </sst>
 </file>
@@ -520,17 +520,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="23.28515625" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="16" max="16" width="45.140625" customWidth="1"/>
+    <col min="1" max="2" width="23.26953125" customWidth="1"/>
+    <col min="3" max="3" width="19.26953125" customWidth="1"/>
+    <col min="5" max="5" width="12.7265625" customWidth="1"/>
+    <col min="16" max="16" width="45.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -539,78 +539,78 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="T1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" s="1" t="s">
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" t="s">
-        <v>20</v>
-      </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D2">
         <v>5.7</v>
       </c>
       <c r="J2">
-        <v>0.43</v>
+        <v>4.3E-3</v>
       </c>
       <c r="M2">
         <v>0.6</v>
@@ -622,36 +622,36 @@
         <v>0.84199999999999997</v>
       </c>
       <c r="P2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="Q2">
         <v>32</v>
       </c>
       <c r="R2" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="S2" t="s">
+        <v>9</v>
+      </c>
+      <c r="U2" t="s">
         <v>19</v>
       </c>
-      <c r="U2" t="s">
-        <v>29</v>
-      </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="D3">
         <v>7.6</v>
       </c>
       <c r="J3">
-        <v>1.04</v>
+        <v>1.04E-2</v>
       </c>
       <c r="M3">
         <v>1.35</v>
@@ -663,36 +663,36 @@
         <v>0.82499999999999996</v>
       </c>
       <c r="P3" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="Q3">
         <v>32</v>
       </c>
       <c r="R3" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="S3" t="s">
+        <v>9</v>
+      </c>
+      <c r="U3" t="s">
         <v>19</v>
       </c>
-      <c r="U3" t="s">
-        <v>29</v>
-      </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="D4">
         <v>7.1</v>
       </c>
       <c r="J4">
-        <v>1.57</v>
+        <v>1.5699999999999999E-2</v>
       </c>
       <c r="M4">
         <v>1.1200000000000001</v>
@@ -704,36 +704,36 @@
         <v>0.89300000000000002</v>
       </c>
       <c r="P4" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="Q4">
         <v>32</v>
       </c>
       <c r="R4" t="s">
+        <v>13</v>
+      </c>
+      <c r="S4" t="s">
+        <v>9</v>
+      </c>
+      <c r="U4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
         <v>23</v>
-      </c>
-      <c r="S4" t="s">
-        <v>19</v>
-      </c>
-      <c r="U4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" t="s">
-        <v>33</v>
       </c>
       <c r="D5">
         <v>7.7</v>
       </c>
       <c r="J5">
-        <v>1.39</v>
+        <v>1.3899999999999999E-2</v>
       </c>
       <c r="M5">
         <v>1.69</v>
@@ -745,36 +745,36 @@
         <v>0.83499999999999996</v>
       </c>
       <c r="P5" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="Q5">
         <v>32</v>
       </c>
       <c r="R5" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="S5" t="s">
+        <v>9</v>
+      </c>
+      <c r="U5" t="s">
         <v>19</v>
       </c>
-      <c r="U5" t="s">
-        <v>29</v>
-      </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D6">
         <v>7.1</v>
       </c>
       <c r="J6">
-        <v>4.3899999999999997</v>
+        <v>4.3900000000000002E-2</v>
       </c>
       <c r="M6">
         <v>3.13</v>
@@ -786,19 +786,19 @@
         <v>0.90700000000000003</v>
       </c>
       <c r="P6" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="Q6">
         <v>32</v>
       </c>
       <c r="R6" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="S6" t="s">
+        <v>9</v>
+      </c>
+      <c r="U6" t="s">
         <v>19</v>
-      </c>
-      <c r="U6" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revise soil sorption table, add some soil sorption and degradation data
- Chemical entities Fluroxypyr-meptyl, MCPA and MCPA-sodium were added
- The `soil_sorption` table was revised to be able to include mean values and to be able to record the type of mean value (geometric or arithmetic). The Freundlich exponent is now recorded as `one_over_n`, and `n` is now the number of values averaged in case a mean value is given.
- Soil sorption and degradation data for the following compounds were added

Ferric phosphate
Fluroxypyr
Fluroxypyr-meptyl
Halauxifen-methyl
MCPB
MCPB-sodium
Propamocarb
Triclopyr
Triclopyr-butotyl

(Commits squashed and commit message edited by jranke)
</commit_message>
<xml_diff>
--- a/data_generation/06_soil_sorption/acetamiprid_soil_sorption.xlsx
+++ b/data_generation/06_soil_sorption/acetamiprid_soil_sorption.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\06_soil_sorption\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9DF5A32-7623-48E5-AF73-E7F8AA07D377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499BFB4A-F8A4-44C0-8185-98A378FB8050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="410" yWindow="520" windowWidth="28800" windowHeight="15410" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="2660" windowWidth="19380" windowHeight="5620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="40">
   <si>
     <t>soil_type</t>
   </si>
@@ -133,6 +133,18 @@
   </si>
   <si>
     <t>Kfoc</t>
+  </si>
+  <si>
+    <t>one_over_n</t>
+  </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
+    <t>mean_type</t>
+  </si>
+  <si>
+    <t>FALSE</t>
   </si>
 </sst>
 </file>
@@ -176,10 +188,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -519,16 +534,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="23.26953125" customWidth="1"/>
     <col min="3" max="3" width="19.26953125" customWidth="1"/>
     <col min="5" max="5" width="12.7265625" customWidth="1"/>
-    <col min="16" max="16" width="45.1796875" customWidth="1"/>
+    <col min="19" max="19" width="45.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:25" s="1" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -571,32 +586,41 @@
       <c r="N1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -622,22 +646,25 @@
         <v>0.84199999999999997</v>
       </c>
       <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="S2" t="s">
         <v>14</v>
       </c>
-      <c r="Q2">
+      <c r="T2">
         <v>32</v>
       </c>
-      <c r="R2" t="s">
+      <c r="U2" t="s">
         <v>13</v>
       </c>
-      <c r="S2" t="s">
+      <c r="V2" t="s">
         <v>9</v>
       </c>
-      <c r="U2" t="s">
+      <c r="X2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -663,22 +690,25 @@
         <v>0.82499999999999996</v>
       </c>
       <c r="P3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S3" t="s">
         <v>14</v>
       </c>
-      <c r="Q3">
+      <c r="T3">
         <v>32</v>
       </c>
-      <c r="R3" t="s">
+      <c r="U3" t="s">
         <v>13</v>
       </c>
-      <c r="S3" t="s">
+      <c r="V3" t="s">
         <v>9</v>
       </c>
-      <c r="U3" t="s">
+      <c r="X3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -704,22 +734,25 @@
         <v>0.89300000000000002</v>
       </c>
       <c r="P4" t="s">
+        <v>39</v>
+      </c>
+      <c r="S4" t="s">
         <v>14</v>
       </c>
-      <c r="Q4">
+      <c r="T4">
         <v>32</v>
       </c>
-      <c r="R4" t="s">
+      <c r="U4" t="s">
         <v>13</v>
       </c>
-      <c r="S4" t="s">
+      <c r="V4" t="s">
         <v>9</v>
       </c>
-      <c r="U4" t="s">
+      <c r="X4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -745,22 +778,25 @@
         <v>0.83499999999999996</v>
       </c>
       <c r="P5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S5" t="s">
         <v>14</v>
       </c>
-      <c r="Q5">
+      <c r="T5">
         <v>32</v>
       </c>
-      <c r="R5" t="s">
+      <c r="U5" t="s">
         <v>13</v>
       </c>
-      <c r="S5" t="s">
+      <c r="V5" t="s">
         <v>9</v>
       </c>
-      <c r="U5" t="s">
+      <c r="X5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -786,23 +822,26 @@
         <v>0.90700000000000003</v>
       </c>
       <c r="P6" t="s">
+        <v>39</v>
+      </c>
+      <c r="S6" t="s">
         <v>14</v>
       </c>
-      <c r="Q6">
+      <c r="T6">
         <v>32</v>
       </c>
-      <c r="R6" t="s">
+      <c r="U6" t="s">
         <v>13</v>
       </c>
-      <c r="S6" t="s">
+      <c r="V6" t="s">
         <v>9</v>
       </c>
-      <c r="U6" t="s">
+      <c r="X6" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V6">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Y6">
     <sortCondition ref="C2:C6"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>